<commit_message>
xlsx changes text fix
</commit_message>
<xml_diff>
--- a/public/price.xlsx
+++ b/public/price.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\durit\WebstormProjects\perch\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0594B8DB-B21B-4467-A1FB-EFC3931EAFCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E8B301-BF6A-4578-8B13-EE36955ED35F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3060" yWindow="2190" windowWidth="28800" windowHeight="15555" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Сайт" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="218">
   <si>
     <t xml:space="preserve">Базилік                                         </t>
   </si>
@@ -151,42 +151,6 @@
   </si>
   <si>
     <t>Пет-банка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Перець чорний мелений 100г </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Часник  сушений   40/60   гранульований   100г                 </t>
-  </si>
-  <si>
-    <t>Суміш "Десять овочів" 50г</t>
-  </si>
-  <si>
-    <t>Суміш "Грузинська" 70г</t>
-  </si>
-  <si>
-    <t>Суміш "Для фаршу" 70г</t>
-  </si>
-  <si>
-    <t>Паприка копчена мелена 70г</t>
-  </si>
-  <si>
-    <t>Суміш "Для бульйону" 100г</t>
-  </si>
-  <si>
-    <t>Суміш "Для барбекю" 70г</t>
-  </si>
-  <si>
-    <t>Суміш "Для м'яса" 70г</t>
-  </si>
-  <si>
-    <t>Суміш пряноароматична "Для сала по європейськи" 100г</t>
-  </si>
-  <si>
-    <t>Суміш пряноароматична до м'яса "Кавказька"70г</t>
-  </si>
-  <si>
-    <t>Суміш пряноароматична "Домашня ковбаса" 70г</t>
   </si>
   <si>
     <t>Подарунковий набір "Classic"</t>
@@ -644,27 +608,6 @@
   </si>
   <si>
     <t>Суміш "Часникова сіль"</t>
-  </si>
-  <si>
-    <t>Суміш "Для картоплі" 90г</t>
-  </si>
-  <si>
-    <t>Суміш "Для плову" 100г</t>
-  </si>
-  <si>
-    <t>Суміш "Для сала" 80г</t>
-  </si>
-  <si>
-    <t>Суміш "Для свинини" 80г</t>
-  </si>
-  <si>
-    <t>Суміш "Для шашлику" 80г</t>
-  </si>
-  <si>
-    <t>Суміш "Європейська"до курки 100г</t>
-  </si>
-  <si>
-    <t>Суміш "Універсальна" 80г</t>
   </si>
   <si>
     <t>Набір спецій "Подарунок господині"</t>
@@ -727,10 +670,34 @@
     <t>Набір спецій "Maksi"</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Шашлик - 70г &lt;br/&gt; 2. Курка - 100г &lt;br/&gt; 3. Сало Європа - 100г  </t>
-  </si>
-  <si>
     <t>podarunok9banok.jpg</t>
+  </si>
+  <si>
+    <t>1. Перець чорний мелений - 100г &lt;br/&gt; 2. Паприка копчена мелена - 70г &lt;br/&gt;  3. Часник гранульований - 100г &lt;br/&gt;  4. Для плову - 100г &lt;br/&gt;  5. До м'яса Кавказська - 70г &lt;br/&gt;  6. Для картоплі - 90г &lt;br/&gt; 7. Шашлик - 70г &lt;br/&gt; 8. Курка - 100г &lt;br/&gt; 9. Сало Європа - 100г</t>
+  </si>
+  <si>
+    <t>50гр</t>
+  </si>
+  <si>
+    <t>70гр.</t>
+  </si>
+  <si>
+    <t>100гр</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Часник  сушений   40/60   гранульований    </t>
+  </si>
+  <si>
+    <t>Суміш "Європейська" до курки</t>
+  </si>
+  <si>
+    <t>Суміш "Для бульйону"г</t>
+  </si>
+  <si>
+    <t>Суміш пряноароматична "Для сала по європейськи"</t>
+  </si>
+  <si>
+    <t>Суміш пряноароматична "Домашня ковбаса"</t>
   </si>
 </sst>
 </file>
@@ -1765,7 +1732,7 @@
     <row r="3" spans="1:5" ht="46.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:5" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>224</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1773,16 +1740,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C5" s="1">
         <v>579</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>218</v>
+        <v>199</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1790,16 +1757,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="C6" s="1">
         <v>323</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>222</v>
+        <v>203</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1807,16 +1774,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="C7" s="1">
         <v>593</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>218</v>
+        <v>199</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1824,16 +1791,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="C8" s="1">
         <v>349</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>222</v>
+        <v>203</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1841,16 +1808,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>211</v>
+        <v>192</v>
       </c>
       <c r="C9" s="1">
         <v>599</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>218</v>
+        <v>199</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>221</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1858,16 +1825,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>219</v>
+        <v>200</v>
       </c>
       <c r="C10" s="1">
         <v>579</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>218</v>
+        <v>199</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>220</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1875,21 +1842,21 @@
         <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>226</v>
+        <v>207</v>
       </c>
       <c r="C11" s="1">
         <v>725</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>227</v>
+        <v>209</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>228</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>225</v>
+        <v>206</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1903,13 +1870,13 @@
         <v>31</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1923,13 +1890,13 @@
         <v>34</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1943,13 +1910,13 @@
         <v>36</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -1963,13 +1930,13 @@
         <v>31</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1983,13 +1950,13 @@
         <v>36</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -2003,13 +1970,13 @@
         <v>32</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -2023,13 +1990,13 @@
         <v>37</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -2043,13 +2010,13 @@
         <v>34</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -2063,13 +2030,13 @@
         <v>55</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2083,13 +2050,13 @@
         <v>33</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -2103,13 +2070,13 @@
         <v>43</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -2123,13 +2090,13 @@
         <v>41</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -2143,13 +2110,13 @@
         <v>37</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -2163,13 +2130,13 @@
         <v>36</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -2177,19 +2144,19 @@
         <v>22</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="C32" s="1">
         <v>34</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -2197,19 +2164,19 @@
         <v>23</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="C33" s="1">
         <v>40</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2217,19 +2184,19 @@
         <v>24</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="C34" s="1">
         <v>35</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -2237,19 +2204,19 @@
         <v>25</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="C35" s="1">
         <v>37</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -2257,19 +2224,19 @@
         <v>26</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="C36" s="1">
         <v>36</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -2277,19 +2244,19 @@
         <v>27</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="C37" s="1">
         <v>39</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -2297,19 +2264,19 @@
         <v>28</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="C38" s="1">
         <v>35</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2317,19 +2284,19 @@
         <v>29</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="C39" s="1">
         <v>36</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -2337,19 +2304,19 @@
         <v>30</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="C40" s="1">
         <v>35</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2357,19 +2324,19 @@
         <v>31</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="C41" s="1">
         <v>50</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2377,19 +2344,19 @@
         <v>32</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="C42" s="1">
         <v>36</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -2397,19 +2364,19 @@
         <v>33</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="C43" s="1">
         <v>33</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2417,19 +2384,19 @@
         <v>34</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="C44" s="1">
         <v>38</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -2437,19 +2404,19 @@
         <v>35</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="C45" s="1">
         <v>40</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -2457,19 +2424,19 @@
         <v>36</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="C46" s="1">
         <v>37</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -2477,19 +2444,19 @@
         <v>37</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="C47" s="1">
         <v>38</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2497,19 +2464,19 @@
         <v>38</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="C48" s="1">
         <v>36</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -2517,19 +2484,19 @@
         <v>39</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="C49" s="1">
         <v>34</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -2537,19 +2504,19 @@
         <v>40</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="C50" s="1">
         <v>37</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -2557,19 +2524,19 @@
         <v>41</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>223</v>
+        <v>204</v>
       </c>
       <c r="C51" s="1">
         <v>36</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -2583,13 +2550,13 @@
         <v>41</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -2603,13 +2570,13 @@
         <v>43</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -2617,19 +2584,19 @@
         <v>44</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="C54" s="1">
         <v>35</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -2643,13 +2610,13 @@
         <v>35</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -2663,13 +2630,13 @@
         <v>49</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -2683,13 +2650,13 @@
         <v>59</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -2703,13 +2670,13 @@
         <v>45</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -2723,13 +2690,13 @@
         <v>42</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -2743,13 +2710,13 @@
         <v>36</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -2763,13 +2730,13 @@
         <v>37</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -2783,13 +2750,13 @@
         <v>36</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -2803,13 +2770,13 @@
         <v>35</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -2823,13 +2790,13 @@
         <v>43</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -2843,13 +2810,13 @@
         <v>38</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
@@ -2863,13 +2830,13 @@
         <v>36</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -2883,13 +2850,13 @@
         <v>35</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -2903,13 +2870,13 @@
         <v>39</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -2923,13 +2890,13 @@
         <v>32</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -2943,13 +2910,13 @@
         <v>36</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2963,13 +2930,13 @@
         <v>35</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2983,13 +2950,13 @@
         <v>36</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -3003,13 +2970,13 @@
         <v>40</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -3023,13 +2990,13 @@
         <v>38</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -3043,13 +3010,13 @@
         <v>42</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -3063,13 +3030,13 @@
         <v>37</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -3083,13 +3050,13 @@
         <v>40</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
@@ -3103,19 +3070,19 @@
         <v>68</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="C80" s="1">
         <v>67</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="F80" t="s">
-        <v>214</v>
+        <v>195</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -3123,19 +3090,19 @@
         <v>69</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>41</v>
+        <v>213</v>
       </c>
       <c r="C81" s="1">
         <v>60</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="F81" t="s">
-        <v>215</v>
+        <v>195</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
@@ -3143,19 +3110,19 @@
         <v>70</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>204</v>
+        <v>173</v>
       </c>
       <c r="C82" s="1">
         <v>64</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="F82" t="s">
-        <v>214</v>
+        <v>196</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
@@ -3163,19 +3130,19 @@
         <v>71</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>205</v>
+        <v>175</v>
       </c>
       <c r="C83" s="1">
         <v>61</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="F83" t="s">
-        <v>216</v>
+        <v>195</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
@@ -3183,19 +3150,19 @@
         <v>72</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>206</v>
+        <v>177</v>
       </c>
       <c r="C84" s="1">
         <v>60</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="F84" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
@@ -3203,19 +3170,19 @@
         <v>73</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>207</v>
+        <v>178</v>
       </c>
       <c r="C85" s="1">
         <v>54</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="F85" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
@@ -3223,19 +3190,19 @@
         <v>74</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>208</v>
+        <v>179</v>
       </c>
       <c r="C86" s="1">
         <v>56</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="F86" t="s">
-        <v>214</v>
+        <v>197</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -3243,19 +3210,19 @@
         <v>75</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C87" s="1">
         <v>57</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F87" t="s">
-        <v>216</v>
+        <v>195</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
@@ -3263,19 +3230,19 @@
         <v>76</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>210</v>
+        <v>182</v>
       </c>
       <c r="C88" s="1">
         <v>55</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="F88" t="s">
-        <v>213</v>
+        <v>197</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -3283,19 +3250,19 @@
         <v>77</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="C89" s="1">
         <v>54</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="F89" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
@@ -3303,19 +3270,19 @@
         <v>78</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="C90" s="1">
         <v>53</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="F90" t="s">
-        <v>217</v>
+        <v>198</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3323,19 +3290,19 @@
         <v>79</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="C91" s="1">
         <v>55</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="F91" t="s">
-        <v>217</v>
+        <v>198</v>
       </c>
     </row>
     <row r="92" spans="1:6" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3343,19 +3310,19 @@
         <v>80</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="C92" s="1">
         <v>53</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="F92" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -3363,19 +3330,19 @@
         <v>81</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>46</v>
+        <v>215</v>
       </c>
       <c r="C93" s="1">
         <v>56</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="F93" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
@@ -3383,19 +3350,19 @@
         <v>82</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="C94" s="1">
         <v>62</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="F94" t="s">
-        <v>217</v>
+        <v>198</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
@@ -3403,19 +3370,19 @@
         <v>83</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="C95" s="1">
         <v>54</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="F95" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
@@ -3423,19 +3390,19 @@
         <v>84</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>49</v>
+        <v>216</v>
       </c>
       <c r="C96" s="1">
         <v>62</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="F96" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
@@ -3443,19 +3410,19 @@
         <v>85</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="C97" s="1">
         <v>61</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="F97" t="s">
-        <v>217</v>
+        <v>198</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -3463,19 +3430,19 @@
         <v>86</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>51</v>
+        <v>217</v>
       </c>
       <c r="C98" s="1">
         <v>59</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>217</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>